<commit_message>
refactor(scheduling): remove legacy diagnostics and greedy solver
</commit_message>
<xml_diff>
--- a/stage_2_scheduling/output/schedule.xlsx
+++ b/stage_2_scheduling/output/schedule.xlsx
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>44</v>
       </c>
       <c r="D2" t="n">
         <v>7</v>
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
         <v>16</v>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="D6" t="n">
         <v>12</v>
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D11" t="n">
         <v>17</v>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D14" t="n">
         <v>16</v>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
         <v>7</v>
@@ -749,13 +749,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="D16" t="n">
         <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="D17" t="n">
         <v>7</v>
@@ -797,7 +797,7 @@
         <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
         <v>11</v>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D20" t="n">
         <v>12</v>
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
         <v>14</v>
@@ -875,10 +875,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="D22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E22" t="n">
         <v>23</v>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D23" t="n">
         <v>16</v>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D25" t="n">
         <v>7</v>
@@ -986,7 +986,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28">
@@ -1001,10 +1001,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="D28" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E28" t="n">
         <v>23</v>
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="D32" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E32" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33">
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
         <v>12</v>
@@ -1133,7 +1133,7 @@
         <v>12</v>
       </c>
       <c r="E34" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -1151,10 +1151,10 @@
         <v>37</v>
       </c>
       <c r="D35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E35" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36">
@@ -1214,10 +1214,10 @@
         <v>41</v>
       </c>
       <c r="D38" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E38" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39">
@@ -1280,7 +1280,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42">
@@ -1295,10 +1295,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="D42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E42" t="n">
         <v>23</v>
@@ -1316,13 +1316,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D43" t="n">
         <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44">
@@ -1337,13 +1337,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="D44" t="n">
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D45" t="n">
         <v>8</v>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="D46" t="n">
         <v>8</v>
@@ -1400,13 +1400,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
         <v>11</v>
       </c>
       <c r="E47" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="48">
@@ -1421,13 +1421,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="D48" t="n">
         <v>12</v>
       </c>
       <c r="E48" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D49" t="n">
         <v>12</v>
@@ -1463,10 +1463,10 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D50" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E50" t="n">
         <v>23</v>
@@ -1484,10 +1484,10 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="D51" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E51" t="n">
         <v>23</v>
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D52" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E52" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="53">
@@ -1526,13 +1526,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="D53" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E53" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="D54" t="n">
         <v>7</v>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
         <v>16</v>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="D56" t="n">
         <v>7</v>
@@ -1610,13 +1610,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
         <v>16</v>
       </c>
       <c r="E57" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58">
@@ -1627,17 +1627,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D58" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59">
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="D59" t="n">
         <v>7</v>
@@ -1673,13 +1673,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D60" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E60" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61">
@@ -1694,13 +1694,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D61" t="n">
         <v>12</v>
       </c>
       <c r="E61" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62">
@@ -1715,13 +1715,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D62" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E62" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="63">
@@ -1736,13 +1736,13 @@
         </is>
       </c>
       <c r="C63" t="n">
+        <v>37</v>
+      </c>
+      <c r="D63" t="n">
+        <v>15</v>
+      </c>
+      <c r="E63" t="n">
         <v>18</v>
-      </c>
-      <c r="D63" t="n">
-        <v>13</v>
-      </c>
-      <c r="E63" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="64">
@@ -1757,13 +1757,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D64" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E64" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65">
@@ -1778,13 +1778,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D65" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E65" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="66">
@@ -1799,13 +1799,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D66" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E66" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67">
@@ -1820,10 +1820,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="D67" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E67" t="n">
         <v>23</v>
@@ -1837,17 +1837,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D68" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E68" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="69">
@@ -1862,13 +1862,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D69" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E69" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70">
@@ -1883,10 +1883,10 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D70" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E70" t="n">
         <v>23</v>
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D71" t="n">
         <v>7</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="D72" t="n">
         <v>7</v>
@@ -1946,13 +1946,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D73" t="n">
         <v>8</v>
       </c>
       <c r="E73" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="74">
@@ -1967,13 +1967,13 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D74" t="n">
         <v>8</v>
       </c>
       <c r="E74" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75">
@@ -1988,7 +1988,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="D75" t="n">
         <v>10</v>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D77" t="n">
         <v>13</v>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>7</v>
+        <v>59</v>
       </c>
       <c r="D78" t="n">
         <v>15</v>
@@ -2072,10 +2072,10 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="D79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E79" t="n">
         <v>23</v>
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="D80" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E80" t="n">
         <v>23</v>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D82" t="n">
         <v>7</v>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D83" t="n">
         <v>16</v>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>66</v>
+        <v>2</v>
       </c>
       <c r="D84" t="n">
         <v>7</v>
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
         <v>16</v>
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="D87" t="n">
         <v>7</v>
@@ -2261,7 +2261,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D88" t="n">
         <v>12</v>
@@ -2330,7 +2330,7 @@
         <v>16</v>
       </c>
       <c r="E91" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="92">
@@ -2351,7 +2351,7 @@
         <v>16</v>
       </c>
       <c r="E92" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="D96" t="n">
         <v>7</v>
@@ -2450,7 +2450,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D97" t="n">
         <v>16</v>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>7</v>
+        <v>54</v>
       </c>
       <c r="D99" t="n">
         <v>7</v>
@@ -2513,13 +2513,13 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D100" t="n">
         <v>7</v>
       </c>
       <c r="E100" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101">
@@ -2534,13 +2534,13 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D101" t="n">
         <v>8</v>
       </c>
       <c r="E101" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="102">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="D103" t="n">
         <v>12</v>
@@ -2603,7 +2603,7 @@
         <v>12</v>
       </c>
       <c r="E104" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="105">
@@ -2618,13 +2618,13 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="D105" t="n">
         <v>14</v>
       </c>
       <c r="E105" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="106">
@@ -2639,7 +2639,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D106" t="n">
         <v>15</v>
@@ -2660,10 +2660,10 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D107" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E107" t="n">
         <v>23</v>
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D108" t="n">
         <v>16</v>
@@ -2702,13 +2702,13 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="D109" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E109" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="110">
@@ -2723,13 +2723,13 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D110" t="n">
         <v>7</v>
       </c>
       <c r="E110" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="111">
@@ -2747,7 +2747,7 @@
         <v>50</v>
       </c>
       <c r="D111" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E111" t="n">
         <v>23</v>
@@ -2765,13 +2765,13 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="D112" t="n">
         <v>7</v>
       </c>
       <c r="E112" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="113">
@@ -2786,10 +2786,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D113" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E113" t="n">
         <v>23</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
         <v>7</v>
@@ -2876,7 +2876,7 @@
         <v>12</v>
       </c>
       <c r="E117" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="118">
@@ -2897,7 +2897,7 @@
         <v>12</v>
       </c>
       <c r="E118" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="119">
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="D124" t="n">
         <v>20</v>
@@ -3101,7 +3101,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D128" t="n">
         <v>20</v>
@@ -3122,13 +3122,13 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
       </c>
       <c r="E129" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="130">
@@ -3143,7 +3143,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -3164,13 +3164,13 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
       </c>
       <c r="E131" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="132">
@@ -3185,7 +3185,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="D132" t="n">
         <v>8</v>
@@ -3206,13 +3206,13 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D133" t="n">
         <v>8</v>
       </c>
       <c r="E133" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="134">
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D134" t="n">
         <v>11</v>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D137" t="n">
         <v>15</v>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D138" t="n">
         <v>15</v>
@@ -3332,10 +3332,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="D139" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E139" t="n">
         <v>23</v>
@@ -3353,7 +3353,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="D140" t="n">
         <v>16</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="D142" t="n">
         <v>20</v>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D144" t="n">
         <v>15</v>
@@ -3458,13 +3458,13 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
       </c>
       <c r="E145" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="146">
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="D146" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E146" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="147">
@@ -3496,17 +3496,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>BVR</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D147" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E147" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="148">
@@ -3517,17 +3517,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>BVR</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="D148" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E148" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="149">
@@ -3542,13 +3542,13 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="D149" t="n">
+        <v>7</v>
+      </c>
+      <c r="E149" t="n">
         <v>10</v>
-      </c>
-      <c r="E149" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="150">
@@ -3563,13 +3563,13 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="D150" t="n">
+        <v>8</v>
+      </c>
+      <c r="E150" t="n">
         <v>11</v>
-      </c>
-      <c r="E150" t="n">
-        <v>18</v>
       </c>
     </row>
     <row r="151">
@@ -3584,13 +3584,13 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D151" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E151" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="152">
@@ -3605,13 +3605,13 @@
         </is>
       </c>
       <c r="C152" t="n">
+        <v>68</v>
+      </c>
+      <c r="D152" t="n">
+        <v>11</v>
+      </c>
+      <c r="E152" t="n">
         <v>18</v>
-      </c>
-      <c r="D152" t="n">
-        <v>13</v>
-      </c>
-      <c r="E152" t="n">
-        <v>16</v>
       </c>
     </row>
     <row r="153">
@@ -3626,13 +3626,13 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E153" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="154">
@@ -3647,13 +3647,13 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D154" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E154" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="155">
@@ -3668,13 +3668,13 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="D155" t="n">
+        <v>14</v>
+      </c>
+      <c r="E155" t="n">
         <v>17</v>
-      </c>
-      <c r="E155" t="n">
-        <v>23</v>
       </c>
     </row>
     <row r="156">
@@ -3689,13 +3689,13 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D156" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E156" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="157">
@@ -3710,10 +3710,10 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="D157" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E157" t="n">
         <v>23</v>
@@ -3731,13 +3731,13 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D158" t="n">
+        <v>17</v>
+      </c>
+      <c r="E158" t="n">
         <v>20</v>
-      </c>
-      <c r="E158" t="n">
-        <v>23</v>
       </c>
     </row>
     <row r="159">
@@ -3748,17 +3748,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="D159" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E159" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="160">
@@ -3769,17 +3769,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="D160" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E160" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
     </row>
     <row r="161">
@@ -3794,13 +3794,13 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="D161" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E161" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
     </row>
     <row r="162">
@@ -3815,13 +3815,13 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="D162" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E162" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="163">
@@ -3832,17 +3832,17 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="D163" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E163" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="164">
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -3878,13 +3878,13 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="D165" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E165" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="166">
@@ -3899,13 +3899,13 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D166" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E166" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="167">
@@ -3920,13 +3920,13 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D167" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E167" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="168">
@@ -3941,13 +3941,13 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="D168" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E168" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="169">
@@ -3962,10 +3962,10 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="D169" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E169" t="n">
         <v>23</v>
@@ -3983,10 +3983,10 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="D170" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E170" t="n">
         <v>23</v>
@@ -4004,10 +4004,10 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="D171" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E171" t="n">
         <v>23</v>
@@ -4021,17 +4021,17 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E172" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="173">
@@ -4046,34 +4046,34 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D173" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E173" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="D174" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E174" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="175">
@@ -4088,13 +4088,13 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="D175" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E175" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="176">
@@ -4109,10 +4109,10 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="D176" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E176" t="n">
         <v>23</v>
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D185" t="n">
         <v>20</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="D186" t="n">
         <v>7</v>
@@ -4340,13 +4340,13 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="D187" t="n">
         <v>16</v>
       </c>
       <c r="E187" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="188">
@@ -4357,17 +4357,17 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="D188" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E188" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="189">
@@ -4382,13 +4382,13 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D189" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E189" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="190">
@@ -4403,13 +4403,13 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="D190" t="n">
+        <v>8</v>
+      </c>
+      <c r="E190" t="n">
         <v>11</v>
-      </c>
-      <c r="E190" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="191">
@@ -4445,13 +4445,13 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="D192" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E192" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="193">
@@ -4466,13 +4466,13 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D193" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E193" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="194">
@@ -4487,10 +4487,10 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D194" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E194" t="n">
         <v>23</v>
@@ -4508,10 +4508,10 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="D195" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E195" t="n">
         <v>23</v>
@@ -4525,17 +4525,17 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="D196" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="E196" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="197">
@@ -4550,13 +4550,13 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="D197" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E197" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="198">
@@ -4574,7 +4574,7 @@
         <v>67</v>
       </c>
       <c r="D198" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E198" t="n">
         <v>17</v>
@@ -4613,7 +4613,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D200" t="n">
         <v>20</v>

</xml_diff>

<commit_message>
style(hero): remove orange footer banner from landing page
</commit_message>
<xml_diff>
--- a/stage_2_scheduling/output/schedule.xlsx
+++ b/stage_2_scheduling/output/schedule.xlsx
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>19</v>
+        <v>59</v>
       </c>
       <c r="D2" t="n">
         <v>7</v>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
         <v>16</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
         <v>7</v>
@@ -770,13 +770,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
         <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
@@ -797,7 +797,7 @@
         <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -896,10 +896,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="D23" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E23" t="n">
         <v>23</v>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="D24" t="n">
         <v>15</v>
@@ -938,10 +938,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="D25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E25" t="n">
         <v>23</v>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D26" t="n">
         <v>16</v>
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>54</v>
+        <v>7</v>
       </c>
       <c r="D27" t="n">
         <v>7</v>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D28" t="n">
         <v>16</v>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D29" t="n">
         <v>7</v>
@@ -1064,13 +1064,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D31" t="n">
         <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32">
@@ -1085,13 +1085,13 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D32" t="n">
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D34" t="n">
         <v>11</v>
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D35" t="n">
         <v>12</v>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D36" t="n">
         <v>12</v>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="D40" t="n">
         <v>17</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="D44" t="n">
         <v>7</v>
@@ -1379,13 +1379,13 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D46" t="n">
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47">
@@ -1400,13 +1400,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D47" t="n">
         <v>7</v>
       </c>
       <c r="E47" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48">
@@ -1421,13 +1421,13 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="D48" t="n">
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D49" t="n">
         <v>8</v>
@@ -1484,13 +1484,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
         <v>12</v>
       </c>
       <c r="E51" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52">
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>12</v>
       </c>
       <c r="E52" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53">
@@ -1526,10 +1526,10 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D53" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E53" t="n">
         <v>23</v>
@@ -1547,10 +1547,10 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D54" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E54" t="n">
         <v>23</v>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D56" t="n">
         <v>18</v>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D57" t="n">
         <v>20</v>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="D58" t="n">
         <v>7</v>
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="D59" t="n">
         <v>15</v>
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D62" t="n">
         <v>7</v>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D65" t="n">
         <v>12</v>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="D66" t="n">
         <v>12</v>
@@ -1946,13 +1946,13 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="D73" t="n">
         <v>7</v>
       </c>
       <c r="E73" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="74">
@@ -1967,10 +1967,10 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D74" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E74" t="n">
         <v>23</v>
@@ -1988,13 +1988,13 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D75" t="n">
         <v>7</v>
       </c>
       <c r="E75" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="76">
@@ -2009,13 +2009,13 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D76" t="n">
         <v>7</v>
       </c>
       <c r="E76" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="77">
@@ -2030,13 +2030,13 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="D77" t="n">
         <v>7</v>
       </c>
       <c r="E77" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="78">
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D78" t="n">
         <v>8</v>
@@ -2093,13 +2093,13 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D80" t="n">
         <v>12</v>
       </c>
       <c r="E80" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="81">
@@ -2114,13 +2114,13 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D81" t="n">
         <v>13</v>
       </c>
       <c r="E81" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="82">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="D82" t="n">
         <v>15</v>
@@ -2156,10 +2156,10 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D83" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E83" t="n">
         <v>23</v>
@@ -2177,10 +2177,10 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D84" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E84" t="n">
         <v>23</v>
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D85" t="n">
         <v>16</v>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D86" t="n">
         <v>17</v>
@@ -2240,13 +2240,13 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="D87" t="n">
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="88">
@@ -2261,10 +2261,10 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E88" t="n">
         <v>23</v>
@@ -2282,7 +2282,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D89" t="n">
         <v>7</v>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
         <v>16</v>
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D93" t="n">
         <v>11</v>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D94" t="n">
         <v>12</v>
@@ -2576,13 +2576,13 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
       </c>
       <c r="E103" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104">
@@ -2597,10 +2597,10 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D104" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E104" t="n">
         <v>23</v>
@@ -2624,7 +2624,7 @@
         <v>7</v>
       </c>
       <c r="E105" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="106">
@@ -2639,13 +2639,13 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D106" t="n">
         <v>7</v>
       </c>
       <c r="E106" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="107">
@@ -2666,7 +2666,7 @@
         <v>7</v>
       </c>
       <c r="E107" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="108">
@@ -2687,7 +2687,7 @@
         <v>8</v>
       </c>
       <c r="E108" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="109">
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="D112" t="n">
         <v>14</v>
@@ -2789,7 +2789,7 @@
         <v>7</v>
       </c>
       <c r="D113" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E113" t="n">
         <v>23</v>
@@ -2807,10 +2807,10 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="D114" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E114" t="n">
         <v>23</v>
@@ -2828,10 +2828,10 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D115" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E115" t="n">
         <v>23</v>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="D116" t="n">
         <v>16</v>
@@ -2891,13 +2891,13 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
       </c>
       <c r="E118" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="119">
@@ -2912,10 +2912,10 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="D119" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E119" t="n">
         <v>23</v>
@@ -2933,13 +2933,13 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
       </c>
       <c r="E120" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="121">
@@ -2954,10 +2954,10 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D121" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E121" t="n">
         <v>23</v>
@@ -2975,7 +2975,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D123" t="n">
         <v>8</v>
@@ -3017,7 +3017,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="D124" t="n">
         <v>12</v>
@@ -3038,7 +3038,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D125" t="n">
         <v>14</v>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -3311,7 +3311,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D139" t="n">
         <v>10</v>
@@ -3395,7 +3395,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D142" t="n">
         <v>14</v>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
         <v>15</v>
@@ -3521,7 +3521,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -3584,13 +3584,13 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
       </c>
       <c r="E151" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="152">
@@ -3605,13 +3605,13 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="D152" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E152" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
     </row>
     <row r="153">
@@ -3622,17 +3622,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D153" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E153" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="154">
@@ -3650,10 +3650,10 @@
         <v>13</v>
       </c>
       <c r="D154" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E154" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="155">
@@ -3668,13 +3668,13 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D155" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E155" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="156">
@@ -3689,13 +3689,13 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="D156" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E156" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="157">
@@ -3710,13 +3710,13 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="D157" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E157" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="158">
@@ -3731,13 +3731,13 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="D158" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E158" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="159">
@@ -3752,7 +3752,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="D159" t="n">
         <v>13</v>
@@ -3773,13 +3773,13 @@
         </is>
       </c>
       <c r="C160" t="n">
+        <v>25</v>
+      </c>
+      <c r="D160" t="n">
+        <v>15</v>
+      </c>
+      <c r="E160" t="n">
         <v>18</v>
-      </c>
-      <c r="D160" t="n">
-        <v>13</v>
-      </c>
-      <c r="E160" t="n">
-        <v>17</v>
       </c>
     </row>
     <row r="161">
@@ -3794,13 +3794,13 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D161" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E161" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
     </row>
     <row r="162">
@@ -3815,13 +3815,13 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D162" t="n">
         <v>17</v>
       </c>
       <c r="E162" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="163">
@@ -3836,13 +3836,13 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="D163" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E163" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="164">
@@ -3857,13 +3857,13 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="D164" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E164" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="165">
@@ -3878,10 +3878,10 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="D165" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E165" t="n">
         <v>23</v>
@@ -3895,17 +3895,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D166" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E166" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="167">
@@ -3920,13 +3920,13 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D167" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E167" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="168">
@@ -3941,13 +3941,13 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="D168" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E168" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="169">
@@ -3962,13 +3962,13 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="D169" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E169" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="170">
@@ -3979,17 +3979,17 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D170" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E170" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="171">
@@ -4004,7 +4004,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -4025,13 +4025,13 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="D172" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E172" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="173">
@@ -4046,13 +4046,13 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D173" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E173" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="174">
@@ -4067,13 +4067,13 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="D174" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E174" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="175">
@@ -4091,7 +4091,7 @@
         <v>56</v>
       </c>
       <c r="D175" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E175" t="n">
         <v>20</v>
@@ -4109,13 +4109,13 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="D176" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E176" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="177">
@@ -4130,10 +4130,10 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="D177" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E177" t="n">
         <v>23</v>
@@ -4151,7 +4151,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D178" t="n">
         <v>15</v>
@@ -4172,7 +4172,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="D179" t="n">
         <v>15</v>
@@ -4193,7 +4193,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="D180" t="n">
         <v>16</v>
@@ -4210,17 +4210,17 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D181" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E181" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="182">
@@ -4235,13 +4235,13 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="D182" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E182" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="183">
@@ -4256,13 +4256,13 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="D183" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E183" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="184">
@@ -4277,10 +4277,10 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="D184" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E184" t="n">
         <v>23</v>
@@ -4289,22 +4289,22 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>BVR</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="E185" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="186">
@@ -4319,13 +4319,13 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="D186" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="E186" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="187">
@@ -4336,17 +4336,17 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="D187" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E187" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="188">
@@ -4357,17 +4357,17 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="D188" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E188" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="189">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>BVR</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="D189" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="E189" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="190">
@@ -4403,13 +4403,13 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D190" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E190" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="191">
@@ -4424,13 +4424,13 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="D191" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E191" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="192">
@@ -4445,13 +4445,13 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="D192" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E192" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="193">
@@ -4466,13 +4466,13 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D193" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E193" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="194">
@@ -4487,13 +4487,13 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D194" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E194" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="195">
@@ -4508,13 +4508,13 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="D195" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E195" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="196">
@@ -4529,13 +4529,13 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D196" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E196" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="197">
@@ -4550,13 +4550,13 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="D197" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E197" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="198">
@@ -4567,17 +4567,17 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="D198" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E198" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="199">
@@ -4588,14 +4588,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D199" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E199" t="n">
         <v>23</v>
@@ -4609,17 +4609,17 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D200" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E200" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="201">
@@ -4630,17 +4630,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D201" t="n">
         <v>7</v>
       </c>
       <c r="E201" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="202">
@@ -4651,17 +4651,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>K</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D202" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E202" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="203">
@@ -4676,13 +4676,13 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="D203" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E203" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="204">
@@ -4697,13 +4697,13 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="D204" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E204" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="205">
@@ -4718,13 +4718,13 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D205" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E205" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="206">
@@ -4739,13 +4739,13 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="D206" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E206" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="207">
@@ -4760,13 +4760,13 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D207" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E207" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="208">
@@ -4781,10 +4781,10 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D208" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E208" t="n">
         <v>23</v>
@@ -4802,10 +4802,10 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D209" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E209" t="n">
         <v>23</v>
@@ -4819,17 +4819,17 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="D210" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="E210" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="211">
@@ -4840,17 +4840,17 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D211" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E211" t="n">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="212">
@@ -4861,17 +4861,17 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>TS</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="D212" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E212" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="213">
@@ -4886,13 +4886,13 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D213" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E213" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="214">
@@ -4907,13 +4907,13 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="D214" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E214" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="215">
@@ -4928,13 +4928,13 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D215" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E215" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>